<commit_message>
slutspel plus kap verde
</commit_message>
<xml_diff>
--- a/Allas tips excel/Anders_F_VM_Tips_2026_AF.xlsx
+++ b/Allas tips excel/Anders_F_VM_Tips_2026_AF.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\VM2026\Allas tips excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5082EC74-10E2-4355-9E72-154C3A5EFC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA07255D-69E6-4D42-A273-02D2F8C55FCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2730" yWindow="1800" windowWidth="25455" windowHeight="14400" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-26235" yWindow="300" windowWidth="25455" windowHeight="15135" firstSheet="3" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instruktion" sheetId="1" r:id="rId1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6075" uniqueCount="932">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6076" uniqueCount="933">
   <si>
     <t>Fält</t>
   </si>
@@ -2966,6 +2966,9 @@
   </si>
   <si>
     <t>Anders Fred</t>
+  </si>
+  <si>
+    <t>Brons</t>
   </si>
 </sst>
 </file>
@@ -3791,7 +3794,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="5"/>
   </cellStyleXfs>
-  <cellXfs count="221">
+  <cellXfs count="223">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4279,11 +4282,23 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="58" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="58" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="58" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4305,15 +4320,6 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="57" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="58" borderId="32" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="58" borderId="33" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="58" borderId="34" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4369,6 +4375,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4971,10 +4978,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="201" t="s">
+      <c r="A1" s="202" t="s">
         <v>919</v>
       </c>
-      <c r="B1" s="202"/>
+      <c r="B1" s="203"/>
       <c r="C1" s="111"/>
       <c r="D1" s="111"/>
       <c r="E1" s="111"/>
@@ -5062,52 +5069,55 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:AH21"/>
+  <dimension ref="A1:AI21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="34" width="15" customWidth="1"/>
+    <col min="2" max="32" width="15" customWidth="1"/>
+    <col min="33" max="33" width="15" style="222" customWidth="1"/>
+    <col min="34" max="35" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A1" s="219" t="s">
+    <row r="1" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A1" s="220" t="s">
         <v>875</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="204"/>
-      <c r="G1" s="204"/>
-      <c r="H1" s="204"/>
-      <c r="I1" s="204"/>
-      <c r="J1" s="204"/>
-      <c r="K1" s="204"/>
-      <c r="L1" s="204"/>
-      <c r="M1" s="204"/>
-      <c r="N1" s="204"/>
-      <c r="O1" s="204"/>
-      <c r="P1" s="204"/>
-      <c r="Q1" s="204"/>
-      <c r="R1" s="204"/>
-      <c r="S1" s="204"/>
-      <c r="T1" s="204"/>
-      <c r="U1" s="204"/>
-      <c r="V1" s="204"/>
-      <c r="W1" s="204"/>
-      <c r="X1" s="204"/>
-      <c r="Y1" s="204"/>
-      <c r="Z1" s="204"/>
-      <c r="AA1" s="204"/>
-      <c r="AB1" s="204"/>
-      <c r="AC1" s="204"/>
-      <c r="AD1" s="204"/>
-      <c r="AE1" s="204"/>
-      <c r="AF1" s="204"/>
-      <c r="AG1" s="204"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
+      <c r="F1" s="205"/>
+      <c r="G1" s="205"/>
+      <c r="H1" s="205"/>
+      <c r="I1" s="205"/>
+      <c r="J1" s="205"/>
+      <c r="K1" s="205"/>
+      <c r="L1" s="205"/>
+      <c r="M1" s="205"/>
+      <c r="N1" s="205"/>
+      <c r="O1" s="205"/>
+      <c r="P1" s="205"/>
+      <c r="Q1" s="205"/>
+      <c r="R1" s="205"/>
+      <c r="S1" s="205"/>
+      <c r="T1" s="205"/>
+      <c r="U1" s="205"/>
+      <c r="V1" s="205"/>
+      <c r="W1" s="205"/>
+      <c r="X1" s="205"/>
+      <c r="Y1" s="205"/>
+      <c r="Z1" s="205"/>
+      <c r="AA1" s="205"/>
+      <c r="AB1" s="205"/>
+      <c r="AC1" s="205"/>
+      <c r="AD1" s="205"/>
+      <c r="AE1" s="205"/>
+      <c r="AF1" s="205"/>
+      <c r="AG1" s="205"/>
       <c r="AH1" s="205"/>
-    </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="AI1" s="206"/>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>876</v>
       </c>
@@ -5204,14 +5214,17 @@
       <c r="AF2" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="AG2" s="1" t="s">
+      <c r="AG2" s="189" t="s">
+        <v>932</v>
+      </c>
+      <c r="AH2" s="1" t="s">
         <v>907</v>
       </c>
-      <c r="AH2" s="1" t="s">
+      <c r="AI2" s="1" t="s">
         <v>908</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="str">
         <f>Instruktion!B10</f>
         <v>Anders Fred</v>
@@ -5341,23 +5354,26 @@
         <v>Spanien</v>
       </c>
       <c r="AG3" s="2" t="str">
+        <f>'3. Slutspelsträd'!Q39</f>
+        <v>Frankrike</v>
+      </c>
+      <c r="AH3" s="2" t="str">
         <f>'4. Skyttekung och utslagsfråga'!C4</f>
         <v>Kai Havertz</v>
       </c>
-      <c r="AH3" s="2">
-        <f>'4. Skyttekung och utslagsfråga'!C6</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A6" s="220" t="s">
+      <c r="AI3" s="2">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="6" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A6" s="221" t="s">
         <v>909</v>
       </c>
-      <c r="B6" s="204"/>
-      <c r="C6" s="204"/>
-      <c r="D6" s="205"/>
-    </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+      <c r="B6" s="205"/>
+      <c r="C6" s="205"/>
+      <c r="D6" s="206"/>
+    </row>
+    <row r="7" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
@@ -5371,7 +5387,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -5388,7 +5404,7 @@
         <v>Tjeckien</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>26</v>
       </c>
@@ -5405,7 +5421,7 @@
         <v>Bosnien och Hercegovina</v>
       </c>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -5422,7 +5438,7 @@
         <v>Marocko</v>
       </c>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
@@ -5439,7 +5455,7 @@
         <v>Paraguay</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>34</v>
       </c>
@@ -5456,7 +5472,7 @@
         <v>Ecuador</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
@@ -5473,7 +5489,7 @@
         <v>Japan</v>
       </c>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>40</v>
       </c>
@@ -5490,7 +5506,7 @@
         <v>Iran</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>43</v>
       </c>
@@ -5507,7 +5523,7 @@
         <v>Uruguay</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>46</v>
       </c>
@@ -5585,7 +5601,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:AH1"/>
+    <mergeCell ref="A1:AI1"/>
     <mergeCell ref="A6:D6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5605,29 +5621,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="204" t="s">
         <v>293</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="205"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
+      <c r="F1" s="206"/>
       <c r="G1" s="85"/>
       <c r="H1" s="34"/>
       <c r="I1" s="34"/>
       <c r="J1" s="34"/>
     </row>
     <row r="2" spans="1:11" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="212" t="s">
+      <c r="A2" s="213" t="s">
         <v>929</v>
       </c>
-      <c r="B2" s="212"/>
-      <c r="C2" s="212"/>
-      <c r="D2" s="212"/>
-      <c r="E2" s="212"/>
-      <c r="F2" s="212"/>
-      <c r="G2" s="212"/>
+      <c r="B2" s="213"/>
+      <c r="C2" s="213"/>
+      <c r="D2" s="213"/>
+      <c r="E2" s="213"/>
+      <c r="F2" s="213"/>
+      <c r="G2" s="213"/>
       <c r="H2" s="54"/>
       <c r="I2" s="54"/>
     </row>
@@ -6397,20 +6413,20 @@
       <c r="G58" s="112"/>
     </row>
     <row r="59" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B59" s="209" t="s">
+      <c r="B59" s="210" t="s">
         <v>922</v>
       </c>
-      <c r="C59" s="210"/>
-      <c r="D59" s="210"/>
-      <c r="E59" s="211"/>
+      <c r="C59" s="211"/>
+      <c r="D59" s="211"/>
+      <c r="E59" s="212"/>
     </row>
     <row r="60" spans="1:7" s="111" customFormat="1" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="206" t="s">
+      <c r="A60" s="207" t="s">
         <v>312</v>
       </c>
-      <c r="B60" s="207"/>
-      <c r="C60" s="207"/>
-      <c r="D60" s="208"/>
+      <c r="B60" s="208"/>
+      <c r="C60" s="208"/>
+      <c r="D60" s="209"/>
     </row>
     <row r="61" spans="1:7" s="111" customFormat="1" ht="14.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="91" t="s">
@@ -6855,24 +6871,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="204" t="s">
         <v>918</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="205"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
+      <c r="F1" s="206"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="213" t="s">
+      <c r="A2" s="214" t="s">
         <v>923</v>
       </c>
-      <c r="B2" s="213"/>
-      <c r="C2" s="213"/>
-      <c r="D2" s="213"/>
-      <c r="E2" s="213"/>
-      <c r="F2" s="213"/>
+      <c r="B2" s="214"/>
+      <c r="C2" s="214"/>
+      <c r="D2" s="214"/>
+      <c r="E2" s="214"/>
+      <c r="F2" s="214"/>
     </row>
     <row r="3" spans="1:6" ht="5.0999999999999996" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6970,11 +6986,11 @@
     </row>
     <row r="19" spans="1:12" ht="9" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:12" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="209" t="s">
+      <c r="B20" s="210" t="s">
         <v>922</v>
       </c>
-      <c r="C20" s="210"/>
-      <c r="D20" s="211"/>
+      <c r="C20" s="211"/>
+      <c r="D20" s="212"/>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="G27" s="177"/>
@@ -7142,32 +7158,32 @@
     </row>
     <row r="3" spans="2:35" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="127"/>
-      <c r="O3" s="192" t="s">
+      <c r="O3" s="196" t="s">
         <v>353</v>
       </c>
-      <c r="P3" s="193"/>
-      <c r="Q3" s="193"/>
-      <c r="R3" s="193"/>
-      <c r="S3" s="194"/>
+      <c r="P3" s="197"/>
+      <c r="Q3" s="197"/>
+      <c r="R3" s="197"/>
+      <c r="S3" s="198"/>
       <c r="AF3" s="128"/>
     </row>
     <row r="4" spans="2:35" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B4" s="127"/>
-      <c r="C4" s="189" t="s">
+      <c r="C4" s="190" t="s">
         <v>914</v>
       </c>
-      <c r="D4" s="189"/>
-      <c r="E4" s="189"/>
-      <c r="O4" s="195"/>
-      <c r="P4" s="196"/>
-      <c r="Q4" s="196"/>
-      <c r="R4" s="196"/>
-      <c r="S4" s="197"/>
-      <c r="AC4" s="189" t="s">
+      <c r="D4" s="190"/>
+      <c r="E4" s="190"/>
+      <c r="O4" s="199"/>
+      <c r="P4" s="200"/>
+      <c r="Q4" s="200"/>
+      <c r="R4" s="200"/>
+      <c r="S4" s="201"/>
+      <c r="AC4" s="190" t="s">
         <v>914</v>
       </c>
-      <c r="AD4" s="189"/>
-      <c r="AE4" s="189"/>
+      <c r="AD4" s="190"/>
+      <c r="AE4" s="190"/>
       <c r="AF4" s="128"/>
     </row>
     <row r="5" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -7208,7 +7224,7 @@
     </row>
     <row r="6" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="127"/>
-      <c r="C6" s="191" t="s">
+      <c r="C6" s="195" t="s">
         <v>251</v>
       </c>
       <c r="D6" s="115" t="str">
@@ -7242,7 +7258,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M76",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Brasilien</v>
       </c>
-      <c r="AE6" s="190" t="s">
+      <c r="AE6" s="191" t="s">
         <v>253</v>
       </c>
       <c r="AF6" s="128"/>
@@ -7252,13 +7268,13 @@
     </row>
     <row r="7" spans="2:35" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B7" s="127"/>
-      <c r="C7" s="191"/>
+      <c r="C7" s="195"/>
       <c r="E7" s="114"/>
-      <c r="F7" s="189" t="s">
+      <c r="F7" s="190" t="s">
         <v>913</v>
       </c>
-      <c r="G7" s="189"/>
-      <c r="H7" s="189"/>
+      <c r="G7" s="190"/>
+      <c r="H7" s="190"/>
       <c r="I7" s="114"/>
       <c r="J7" s="114"/>
       <c r="K7" s="114"/>
@@ -7276,13 +7292,13 @@
       <c r="W7" s="114"/>
       <c r="X7" s="114"/>
       <c r="Y7" s="114"/>
-      <c r="Z7" s="189" t="s">
+      <c r="Z7" s="190" t="s">
         <v>913</v>
       </c>
-      <c r="AA7" s="189"/>
-      <c r="AB7" s="189"/>
+      <c r="AA7" s="190"/>
+      <c r="AB7" s="190"/>
       <c r="AC7" s="114"/>
-      <c r="AE7" s="190"/>
+      <c r="AE7" s="191"/>
       <c r="AF7" s="128"/>
       <c r="AG7" s="119"/>
       <c r="AH7" s="114"/>
@@ -7290,7 +7306,7 @@
     </row>
     <row r="8" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B8" s="127"/>
-      <c r="C8" s="191"/>
+      <c r="C8" s="195"/>
       <c r="D8" s="122" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M74",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Marocko</v>
@@ -7324,7 +7340,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M76",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Sverige</v>
       </c>
-      <c r="AE8" s="190"/>
+      <c r="AE8" s="191"/>
       <c r="AF8" s="128"/>
       <c r="AG8" s="119"/>
       <c r="AH8" s="114"/>
@@ -7335,7 +7351,7 @@
       <c r="C9" s="123"/>
       <c r="D9" s="114"/>
       <c r="E9" s="114"/>
-      <c r="F9" s="190" t="s">
+      <c r="F9" s="191" t="s">
         <v>265</v>
       </c>
       <c r="G9" s="115" t="s">
@@ -7357,7 +7373,7 @@
       <c r="AA9" s="115" t="s">
         <v>75</v>
       </c>
-      <c r="AB9" s="190" t="s">
+      <c r="AB9" s="191" t="s">
         <v>267</v>
       </c>
       <c r="AD9" s="114"/>
@@ -7372,7 +7388,7 @@
       <c r="C10" s="123"/>
       <c r="D10" s="114"/>
       <c r="E10" s="114"/>
-      <c r="F10" s="190"/>
+      <c r="F10" s="191"/>
       <c r="G10" s="114"/>
       <c r="H10" s="114"/>
       <c r="I10" s="114"/>
@@ -7391,7 +7407,7 @@
       <c r="W10" s="120"/>
       <c r="Z10" s="114"/>
       <c r="AA10" s="114"/>
-      <c r="AB10" s="190"/>
+      <c r="AB10" s="191"/>
       <c r="AD10" s="114"/>
       <c r="AE10" s="114"/>
       <c r="AF10" s="130"/>
@@ -7404,7 +7420,7 @@
       <c r="C11" s="123"/>
       <c r="D11" s="114"/>
       <c r="E11" s="114"/>
-      <c r="F11" s="190"/>
+      <c r="F11" s="191"/>
       <c r="G11" s="115" t="s">
         <v>97</v>
       </c>
@@ -7430,7 +7446,7 @@
       <c r="AA11" s="115" t="s">
         <v>95</v>
       </c>
-      <c r="AB11" s="190"/>
+      <c r="AB11" s="191"/>
       <c r="AD11" s="114"/>
       <c r="AE11" s="114"/>
       <c r="AF11" s="130"/>
@@ -7440,7 +7456,7 @@
     </row>
     <row r="12" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="127"/>
-      <c r="C12" s="190" t="s">
+      <c r="C12" s="191" t="s">
         <v>252</v>
       </c>
       <c r="D12" s="115" t="str">
@@ -7469,7 +7485,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M78",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Elfenbenskusten</v>
       </c>
-      <c r="AE12" s="190" t="s">
+      <c r="AE12" s="191" t="s">
         <v>254</v>
       </c>
       <c r="AF12" s="128"/>
@@ -7479,33 +7495,33 @@
     </row>
     <row r="13" spans="2:35" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="127"/>
-      <c r="C13" s="190"/>
+      <c r="C13" s="191"/>
       <c r="D13" s="114"/>
       <c r="E13" s="114"/>
       <c r="F13" s="114"/>
       <c r="G13" s="114"/>
       <c r="H13" s="114"/>
-      <c r="I13" s="189" t="s">
+      <c r="I13" s="190" t="s">
         <v>915</v>
       </c>
-      <c r="J13" s="189"/>
-      <c r="K13" s="189"/>
+      <c r="J13" s="190"/>
+      <c r="K13" s="190"/>
       <c r="L13" s="114"/>
       <c r="M13" s="114"/>
       <c r="N13" s="114"/>
       <c r="T13" s="114"/>
       <c r="U13" s="114"/>
       <c r="V13" s="114"/>
-      <c r="W13" s="189" t="s">
+      <c r="W13" s="190" t="s">
         <v>915</v>
       </c>
-      <c r="X13" s="189"/>
-      <c r="Y13" s="189"/>
+      <c r="X13" s="190"/>
+      <c r="Y13" s="190"/>
       <c r="Z13" s="114"/>
       <c r="AA13" s="114"/>
       <c r="AB13" s="114"/>
       <c r="AC13" s="114"/>
-      <c r="AE13" s="190"/>
+      <c r="AE13" s="191"/>
       <c r="AF13" s="128"/>
       <c r="AG13" s="119"/>
       <c r="AH13" s="114"/>
@@ -7513,7 +7529,7 @@
     </row>
     <row r="14" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B14" s="127"/>
-      <c r="C14" s="190"/>
+      <c r="C14" s="191"/>
       <c r="D14" s="122" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M77",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Japan</v>
@@ -7544,7 +7560,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M78",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Frankrike</v>
       </c>
-      <c r="AE14" s="190"/>
+      <c r="AE14" s="191"/>
       <c r="AF14" s="128"/>
       <c r="AG14" s="119"/>
       <c r="AH14" s="114"/>
@@ -7558,7 +7574,7 @@
       <c r="F15" s="114"/>
       <c r="G15" s="114"/>
       <c r="H15" s="114"/>
-      <c r="I15" s="190" t="s">
+      <c r="I15" s="191" t="s">
         <v>273</v>
       </c>
       <c r="J15" s="115" t="s">
@@ -7577,7 +7593,7 @@
       <c r="X15" s="115" t="s">
         <v>95</v>
       </c>
-      <c r="Y15" s="190" t="s">
+      <c r="Y15" s="191" t="s">
         <v>275</v>
       </c>
       <c r="AA15" s="114"/>
@@ -7598,7 +7614,7 @@
       <c r="F16" s="114"/>
       <c r="G16" s="114"/>
       <c r="H16" s="114"/>
-      <c r="I16" s="190"/>
+      <c r="I16" s="191"/>
       <c r="J16" s="114"/>
       <c r="K16" s="114"/>
       <c r="L16" s="114"/>
@@ -7613,7 +7629,7 @@
       <c r="V16" s="114"/>
       <c r="W16" s="114"/>
       <c r="X16" s="114"/>
-      <c r="Y16" s="190"/>
+      <c r="Y16" s="191"/>
       <c r="AA16" s="114"/>
       <c r="AB16" s="114"/>
       <c r="AC16" s="114"/>
@@ -7632,7 +7648,7 @@
       <c r="F17" s="114"/>
       <c r="G17" s="114"/>
       <c r="H17" s="114"/>
-      <c r="I17" s="190"/>
+      <c r="I17" s="191"/>
       <c r="J17" s="115" t="s">
         <v>71</v>
       </c>
@@ -7651,7 +7667,7 @@
       <c r="X17" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="Y17" s="190"/>
+      <c r="Y17" s="191"/>
       <c r="AA17" s="114"/>
       <c r="AB17" s="114"/>
       <c r="AC17" s="114"/>
@@ -7664,7 +7680,7 @@
     </row>
     <row r="18" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B18" s="127"/>
-      <c r="C18" s="190" t="s">
+      <c r="C18" s="191" t="s">
         <v>249</v>
       </c>
       <c r="D18" s="115" t="str">
@@ -7702,7 +7718,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M79",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Sydkorea</v>
       </c>
-      <c r="AE18" s="190" t="s">
+      <c r="AE18" s="191" t="s">
         <v>255</v>
       </c>
       <c r="AF18" s="128"/>
@@ -7712,7 +7728,7 @@
     </row>
     <row r="19" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B19" s="127"/>
-      <c r="C19" s="190"/>
+      <c r="C19" s="191"/>
       <c r="D19" s="114"/>
       <c r="E19" s="114"/>
       <c r="F19" s="114"/>
@@ -7741,7 +7757,7 @@
       <c r="AA19" s="114"/>
       <c r="AB19" s="114"/>
       <c r="AC19" s="114"/>
-      <c r="AE19" s="190"/>
+      <c r="AE19" s="191"/>
       <c r="AF19" s="128"/>
       <c r="AG19" s="119"/>
       <c r="AH19" s="114"/>
@@ -7749,7 +7765,7 @@
     </row>
     <row r="20" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B20" s="127"/>
-      <c r="C20" s="190"/>
+      <c r="C20" s="191"/>
       <c r="D20" s="115" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M73",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Kanada</v>
@@ -7781,7 +7797,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M79",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Uruguay</v>
       </c>
-      <c r="AE20" s="190"/>
+      <c r="AE20" s="191"/>
       <c r="AF20" s="128"/>
       <c r="AG20" s="119"/>
       <c r="AH20" s="114"/>
@@ -7790,7 +7806,7 @@
     <row r="21" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="127"/>
       <c r="E21" s="114"/>
-      <c r="F21" s="190" t="s">
+      <c r="F21" s="191" t="s">
         <v>266</v>
       </c>
       <c r="G21" s="115" t="s">
@@ -7821,7 +7837,7 @@
       <c r="AA21" s="115" t="s">
         <v>93</v>
       </c>
-      <c r="AB21" s="190" t="s">
+      <c r="AB21" s="191" t="s">
         <v>268</v>
       </c>
       <c r="AD21" s="114"/>
@@ -7834,7 +7850,7 @@
     <row r="22" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="127"/>
       <c r="E22" s="114"/>
-      <c r="F22" s="190"/>
+      <c r="F22" s="191"/>
       <c r="G22" s="114"/>
       <c r="H22" s="114"/>
       <c r="I22" s="114"/>
@@ -7856,7 +7872,7 @@
       <c r="Y22" s="114"/>
       <c r="Z22" s="114"/>
       <c r="AA22" s="114"/>
-      <c r="AB22" s="190"/>
+      <c r="AB22" s="191"/>
       <c r="AD22" s="114"/>
       <c r="AE22" s="114"/>
       <c r="AF22" s="130"/>
@@ -7867,7 +7883,7 @@
     <row r="23" spans="2:35" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B23" s="127"/>
       <c r="E23" s="114"/>
-      <c r="F23" s="190"/>
+      <c r="F23" s="191"/>
       <c r="G23" s="115" t="s">
         <v>71</v>
       </c>
@@ -7879,11 +7895,11 @@
       <c r="M23" s="114"/>
       <c r="N23" s="114"/>
       <c r="O23" s="114"/>
-      <c r="P23" s="189" t="s">
+      <c r="P23" s="190" t="s">
         <v>318</v>
       </c>
-      <c r="Q23" s="189"/>
-      <c r="R23" s="189"/>
+      <c r="Q23" s="190"/>
+      <c r="R23" s="190"/>
       <c r="S23" s="114"/>
       <c r="T23" s="114"/>
       <c r="U23" s="114"/>
@@ -7895,7 +7911,7 @@
       <c r="AA23" s="115" t="s">
         <v>99</v>
       </c>
-      <c r="AB23" s="190"/>
+      <c r="AB23" s="191"/>
       <c r="AD23" s="114"/>
       <c r="AE23" s="114"/>
       <c r="AF23" s="128"/>
@@ -7904,7 +7920,7 @@
     </row>
     <row r="24" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B24" s="127"/>
-      <c r="C24" s="190" t="s">
+      <c r="C24" s="191" t="s">
         <v>250</v>
       </c>
       <c r="D24" s="115" t="str">
@@ -7937,7 +7953,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M80",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>England</v>
       </c>
-      <c r="AE24" s="190" t="s">
+      <c r="AE24" s="191" t="s">
         <v>256</v>
       </c>
       <c r="AF24" s="128"/>
@@ -7947,7 +7963,7 @@
     </row>
     <row r="25" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="127"/>
-      <c r="C25" s="190"/>
+      <c r="C25" s="191"/>
       <c r="D25" s="114"/>
       <c r="E25" s="114"/>
       <c r="F25" s="114"/>
@@ -7972,7 +7988,7 @@
       <c r="AA25" s="114"/>
       <c r="AB25" s="114"/>
       <c r="AC25" s="114"/>
-      <c r="AE25" s="190"/>
+      <c r="AE25" s="191"/>
       <c r="AF25" s="128"/>
       <c r="AG25" s="119"/>
       <c r="AH25" s="114"/>
@@ -7980,7 +7996,7 @@
     </row>
     <row r="26" spans="2:35" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B26" s="127"/>
-      <c r="C26" s="190"/>
+      <c r="C26" s="191"/>
       <c r="D26" s="115" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M75",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Skottland</v>
@@ -7992,23 +8008,23 @@
       <c r="I26" s="114"/>
       <c r="J26" s="114"/>
       <c r="K26" s="114"/>
-      <c r="L26" s="189" t="s">
+      <c r="L26" s="190" t="s">
         <v>916</v>
       </c>
-      <c r="M26" s="189"/>
-      <c r="N26" s="189"/>
+      <c r="M26" s="190"/>
+      <c r="N26" s="190"/>
       <c r="O26" s="114"/>
-      <c r="P26" s="198" t="s">
+      <c r="P26" s="192" t="s">
         <v>922</v>
       </c>
-      <c r="Q26" s="199"/>
-      <c r="R26" s="200"/>
+      <c r="Q26" s="193"/>
+      <c r="R26" s="194"/>
       <c r="S26" s="114"/>
-      <c r="T26" s="189" t="s">
+      <c r="T26" s="190" t="s">
         <v>916</v>
       </c>
-      <c r="U26" s="189"/>
-      <c r="V26" s="189"/>
+      <c r="U26" s="190"/>
+      <c r="V26" s="190"/>
       <c r="W26" s="114"/>
       <c r="Z26" s="114"/>
       <c r="AA26" s="114"/>
@@ -8018,7 +8034,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M80",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Senegal</v>
       </c>
-      <c r="AE26" s="190"/>
+      <c r="AE26" s="191"/>
       <c r="AF26" s="128"/>
       <c r="AG26" s="119"/>
       <c r="AH26" s="114"/>
@@ -8067,7 +8083,7 @@
       <c r="I28" s="114"/>
       <c r="J28" s="114"/>
       <c r="K28" s="114"/>
-      <c r="L28" s="190" t="s">
+      <c r="L28" s="191" t="s">
         <v>277</v>
       </c>
       <c r="M28" s="115" t="s">
@@ -8083,7 +8099,7 @@
       <c r="U28" s="115" t="s">
         <v>95</v>
       </c>
-      <c r="V28" s="190" t="s">
+      <c r="V28" s="191" t="s">
         <v>278</v>
       </c>
       <c r="X28" s="114"/>
@@ -8108,7 +8124,7 @@
       <c r="I29" s="114"/>
       <c r="J29" s="114"/>
       <c r="K29" s="114"/>
-      <c r="L29" s="190"/>
+      <c r="L29" s="191"/>
       <c r="M29" s="114"/>
       <c r="N29" s="114"/>
       <c r="O29" s="114"/>
@@ -8118,7 +8134,7 @@
       <c r="S29" s="114"/>
       <c r="T29" s="114"/>
       <c r="U29" s="114"/>
-      <c r="V29" s="190"/>
+      <c r="V29" s="191"/>
       <c r="Z29" s="114"/>
       <c r="AA29" s="114"/>
       <c r="AB29" s="114"/>
@@ -8139,7 +8155,7 @@
       <c r="I30" s="114"/>
       <c r="J30" s="114"/>
       <c r="K30" s="114"/>
-      <c r="L30" s="190"/>
+      <c r="L30" s="191"/>
       <c r="M30" s="115" t="s">
         <v>91</v>
       </c>
@@ -8153,7 +8169,7 @@
       <c r="U30" s="115" t="s">
         <v>104</v>
       </c>
-      <c r="V30" s="190"/>
+      <c r="V30" s="191"/>
       <c r="X30" s="114"/>
       <c r="Y30" s="114"/>
       <c r="Z30" s="114"/>
@@ -8205,7 +8221,7 @@
     </row>
     <row r="32" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="127"/>
-      <c r="C32" s="190" t="s">
+      <c r="C32" s="191" t="s">
         <v>257</v>
       </c>
       <c r="D32" s="115" t="str">
@@ -8238,7 +8254,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M86",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Argentina</v>
       </c>
-      <c r="AE32" s="190" t="s">
+      <c r="AE32" s="191" t="s">
         <v>261</v>
       </c>
       <c r="AF32" s="128"/>
@@ -8248,7 +8264,7 @@
     </row>
     <row r="33" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="127"/>
-      <c r="C33" s="190"/>
+      <c r="C33" s="191"/>
       <c r="D33" s="114"/>
       <c r="E33" s="114"/>
       <c r="F33" s="114"/>
@@ -8272,7 +8288,7 @@
       <c r="AA33" s="114"/>
       <c r="AB33" s="114"/>
       <c r="AC33" s="114"/>
-      <c r="AE33" s="190"/>
+      <c r="AE33" s="191"/>
       <c r="AF33" s="128"/>
       <c r="AG33" s="119"/>
       <c r="AH33" s="114"/>
@@ -8280,7 +8296,7 @@
     </row>
     <row r="34" spans="2:35" ht="21.75" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B34" s="127"/>
-      <c r="C34" s="190"/>
+      <c r="C34" s="191"/>
       <c r="D34" s="115" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M83",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Kroatien</v>
@@ -8295,11 +8311,11 @@
       <c r="M34" s="114"/>
       <c r="N34" s="114"/>
       <c r="O34" s="114"/>
-      <c r="P34" s="189" t="s">
+      <c r="P34" s="190" t="s">
         <v>917</v>
       </c>
-      <c r="Q34" s="189"/>
-      <c r="R34" s="189"/>
+      <c r="Q34" s="190"/>
+      <c r="R34" s="190"/>
       <c r="S34" s="114"/>
       <c r="T34" s="114"/>
       <c r="U34" s="114"/>
@@ -8315,7 +8331,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M86",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Kap Verde</v>
       </c>
-      <c r="AE34" s="190"/>
+      <c r="AE34" s="191"/>
       <c r="AF34" s="128"/>
       <c r="AG34" s="119"/>
       <c r="AH34" s="114"/>
@@ -8326,7 +8342,7 @@
       <c r="C35" s="114"/>
       <c r="D35" s="114"/>
       <c r="E35" s="114"/>
-      <c r="F35" s="190" t="s">
+      <c r="F35" s="191" t="s">
         <v>269</v>
       </c>
       <c r="G35" s="115" t="s">
@@ -8354,7 +8370,7 @@
       <c r="AA35" s="115" t="s">
         <v>104</v>
       </c>
-      <c r="AB35" s="190" t="s">
+      <c r="AB35" s="191" t="s">
         <v>271</v>
       </c>
       <c r="AD35" s="114"/>
@@ -8369,7 +8385,7 @@
       <c r="C36" s="114"/>
       <c r="D36" s="114"/>
       <c r="E36" s="114"/>
-      <c r="F36" s="190"/>
+      <c r="F36" s="191"/>
       <c r="G36" s="114"/>
       <c r="H36" s="114"/>
       <c r="I36" s="114"/>
@@ -8394,7 +8410,7 @@
       <c r="Y36" s="114"/>
       <c r="Z36" s="114"/>
       <c r="AA36" s="114"/>
-      <c r="AB36" s="190"/>
+      <c r="AB36" s="191"/>
       <c r="AD36" s="114"/>
       <c r="AE36" s="114"/>
       <c r="AF36" s="130"/>
@@ -8405,7 +8421,7 @@
     <row r="37" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="127"/>
       <c r="E37" s="114"/>
-      <c r="F37" s="190"/>
+      <c r="F37" s="191"/>
       <c r="G37" s="115" t="s">
         <v>91</v>
       </c>
@@ -8417,7 +8433,7 @@
       <c r="AA37" s="115" t="s">
         <v>56</v>
       </c>
-      <c r="AB37" s="190"/>
+      <c r="AB37" s="191"/>
       <c r="AE37" s="114"/>
       <c r="AF37" s="128"/>
       <c r="AH37" s="114"/>
@@ -8425,7 +8441,7 @@
     </row>
     <row r="38" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="127"/>
-      <c r="C38" s="190" t="s">
+      <c r="C38" s="191" t="s">
         <v>258</v>
       </c>
       <c r="D38" s="115" t="str">
@@ -8463,7 +8479,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M88",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>USA</v>
       </c>
-      <c r="AE38" s="190" t="s">
+      <c r="AE38" s="191" t="s">
         <v>262</v>
       </c>
       <c r="AF38" s="128"/>
@@ -8473,7 +8489,7 @@
     </row>
     <row r="39" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B39" s="127"/>
-      <c r="C39" s="190"/>
+      <c r="C39" s="191"/>
       <c r="D39" s="114"/>
       <c r="E39" s="114"/>
       <c r="F39" s="114"/>
@@ -8499,7 +8515,7 @@
       <c r="AA39" s="114"/>
       <c r="AB39" s="114"/>
       <c r="AC39" s="114"/>
-      <c r="AE39" s="190"/>
+      <c r="AE39" s="191"/>
       <c r="AF39" s="128"/>
       <c r="AG39" s="119"/>
       <c r="AH39" s="114"/>
@@ -8507,7 +8523,7 @@
     </row>
     <row r="40" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B40" s="127"/>
-      <c r="C40" s="190"/>
+      <c r="C40" s="191"/>
       <c r="D40" s="115" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M84",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Österrike</v>
@@ -8535,7 +8551,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M88",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Egypten</v>
       </c>
-      <c r="AE40" s="190"/>
+      <c r="AE40" s="191"/>
       <c r="AF40" s="128"/>
       <c r="AG40" s="119"/>
       <c r="AH40" s="114"/>
@@ -8549,7 +8565,7 @@
       <c r="F41" s="114"/>
       <c r="G41" s="114"/>
       <c r="H41" s="114"/>
-      <c r="I41" s="190" t="s">
+      <c r="I41" s="191" t="s">
         <v>274</v>
       </c>
       <c r="J41" s="115" t="s">
@@ -8568,7 +8584,7 @@
       <c r="X41" s="115" t="s">
         <v>104</v>
       </c>
-      <c r="Y41" s="190" t="s">
+      <c r="Y41" s="191" t="s">
         <v>276</v>
       </c>
       <c r="AA41" s="114"/>
@@ -8589,7 +8605,7 @@
       <c r="F42" s="114"/>
       <c r="G42" s="114"/>
       <c r="H42" s="114"/>
-      <c r="I42" s="190"/>
+      <c r="I42" s="191"/>
       <c r="J42" s="114"/>
       <c r="K42" s="114"/>
       <c r="L42" s="114"/>
@@ -8605,7 +8621,7 @@
       <c r="V42" s="114"/>
       <c r="W42" s="114"/>
       <c r="X42" s="114"/>
-      <c r="Y42" s="190"/>
+      <c r="Y42" s="191"/>
       <c r="AA42" s="114"/>
       <c r="AB42" s="114"/>
       <c r="AC42" s="114"/>
@@ -8623,7 +8639,7 @@
       <c r="F43" s="114"/>
       <c r="G43" s="114"/>
       <c r="H43" s="114"/>
-      <c r="I43" s="190"/>
+      <c r="I43" s="191"/>
       <c r="J43" s="115" t="s">
         <v>79</v>
       </c>
@@ -8643,7 +8659,7 @@
       <c r="X43" s="115" t="s">
         <v>41</v>
       </c>
-      <c r="Y43" s="190"/>
+      <c r="Y43" s="191"/>
       <c r="AA43" s="114"/>
       <c r="AB43" s="114"/>
       <c r="AC43" s="114"/>
@@ -8655,7 +8671,7 @@
     </row>
     <row r="44" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="127"/>
-      <c r="C44" s="190" t="s">
+      <c r="C44" s="191" t="s">
         <v>259</v>
       </c>
       <c r="D44" s="115" t="str">
@@ -8691,7 +8707,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M85",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Schweiz</v>
       </c>
-      <c r="AE44" s="190" t="s">
+      <c r="AE44" s="191" t="s">
         <v>263</v>
       </c>
       <c r="AF44" s="128"/>
@@ -8701,7 +8717,7 @@
     </row>
     <row r="45" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B45" s="127"/>
-      <c r="C45" s="190"/>
+      <c r="C45" s="191"/>
       <c r="D45" s="114"/>
       <c r="E45" s="114"/>
       <c r="G45" s="114"/>
@@ -8727,7 +8743,7 @@
       <c r="AA45" s="114"/>
       <c r="AB45" s="114"/>
       <c r="AC45" s="114"/>
-      <c r="AE45" s="190"/>
+      <c r="AE45" s="191"/>
       <c r="AF45" s="128"/>
       <c r="AG45" s="119"/>
       <c r="AH45" s="114"/>
@@ -8735,7 +8751,7 @@
     </row>
     <row r="46" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="127"/>
-      <c r="C46" s="190"/>
+      <c r="C46" s="191"/>
       <c r="D46" s="122" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M81",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Bosnien och Hercegovina</v>
@@ -8769,7 +8785,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M85",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Iran</v>
       </c>
-      <c r="AE46" s="190"/>
+      <c r="AE46" s="191"/>
       <c r="AF46" s="128"/>
       <c r="AG46" s="119"/>
       <c r="AH46" s="114"/>
@@ -8779,7 +8795,7 @@
       <c r="B47" s="127"/>
       <c r="D47" s="114"/>
       <c r="E47" s="114"/>
-      <c r="F47" s="190" t="s">
+      <c r="F47" s="191" t="s">
         <v>270</v>
       </c>
       <c r="G47" s="115" t="s">
@@ -8807,7 +8823,7 @@
       <c r="AA47" s="115" t="s">
         <v>41</v>
       </c>
-      <c r="AB47" s="190" t="s">
+      <c r="AB47" s="191" t="s">
         <v>272</v>
       </c>
       <c r="AD47" s="114"/>
@@ -8819,7 +8835,7 @@
       <c r="B48" s="127"/>
       <c r="D48" s="114"/>
       <c r="E48" s="114"/>
-      <c r="F48" s="190"/>
+      <c r="F48" s="191"/>
       <c r="G48" s="114"/>
       <c r="H48" s="114"/>
       <c r="I48" s="114"/>
@@ -8841,7 +8857,7 @@
       <c r="Y48" s="114"/>
       <c r="Z48" s="114"/>
       <c r="AA48" s="114"/>
-      <c r="AB48" s="190"/>
+      <c r="AB48" s="191"/>
       <c r="AD48" s="114"/>
       <c r="AF48" s="130"/>
       <c r="AG48" s="114"/>
@@ -8853,7 +8869,7 @@
       <c r="C49" s="114"/>
       <c r="D49" s="114"/>
       <c r="E49" s="114"/>
-      <c r="F49" s="190"/>
+      <c r="F49" s="191"/>
       <c r="G49" s="115" t="s">
         <v>79</v>
       </c>
@@ -8879,7 +8895,7 @@
       <c r="AA49" s="115" t="s">
         <v>114</v>
       </c>
-      <c r="AB49" s="190"/>
+      <c r="AB49" s="191"/>
       <c r="AD49" s="114"/>
       <c r="AF49" s="130"/>
       <c r="AG49" s="114"/>
@@ -8888,7 +8904,7 @@
     </row>
     <row r="50" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="127"/>
-      <c r="C50" s="190" t="s">
+      <c r="C50" s="191" t="s">
         <v>260</v>
       </c>
       <c r="D50" s="115" t="str">
@@ -8924,7 +8940,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M87",_Listor!$BX$3:$BX$18,0),1)</f>
         <v>Portugal</v>
       </c>
-      <c r="AE50" s="190" t="s">
+      <c r="AE50" s="191" t="s">
         <v>264</v>
       </c>
       <c r="AF50" s="128"/>
@@ -8934,7 +8950,7 @@
     </row>
     <row r="51" spans="2:35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="127"/>
-      <c r="C51" s="190"/>
+      <c r="C51" s="191"/>
       <c r="D51" s="114"/>
       <c r="E51" s="114"/>
       <c r="F51" s="114"/>
@@ -8961,7 +8977,7 @@
       <c r="AA51" s="114"/>
       <c r="AB51" s="114"/>
       <c r="AC51" s="114"/>
-      <c r="AE51" s="190"/>
+      <c r="AE51" s="191"/>
       <c r="AF51" s="128"/>
       <c r="AG51" s="119"/>
       <c r="AH51" s="114"/>
@@ -8969,7 +8985,7 @@
     </row>
     <row r="52" spans="2:35" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B52" s="127"/>
-      <c r="C52" s="190"/>
+      <c r="C52" s="191"/>
       <c r="D52" s="122" t="str">
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M82",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Tjeckien</v>
@@ -9003,7 +9019,7 @@
         <f>INDEX(_Listor!$BY$3:$BZ$18,MATCH("M87",_Listor!$BX$3:$BX$18,0),2)</f>
         <v>Paraguay</v>
       </c>
-      <c r="AE52" s="190"/>
+      <c r="AE52" s="191"/>
       <c r="AF52" s="128"/>
       <c r="AG52" s="119"/>
       <c r="AH52" s="114"/>
@@ -9047,21 +9063,17 @@
     </row>
   </sheetData>
   <mergeCells count="42">
-    <mergeCell ref="P34:R34"/>
-    <mergeCell ref="T26:V26"/>
-    <mergeCell ref="L28:L30"/>
-    <mergeCell ref="I41:I43"/>
-    <mergeCell ref="I15:I17"/>
-    <mergeCell ref="AC4:AE4"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="Y41:Y43"/>
-    <mergeCell ref="Y15:Y17"/>
-    <mergeCell ref="V28:V30"/>
-    <mergeCell ref="C50:C52"/>
-    <mergeCell ref="C44:C46"/>
-    <mergeCell ref="C38:C40"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="L26:N26"/>
+    <mergeCell ref="P23:R23"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="C6:C8"/>
+    <mergeCell ref="F9:F11"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="O3:S4"/>
+    <mergeCell ref="F21:F23"/>
     <mergeCell ref="F35:F37"/>
     <mergeCell ref="AE50:AE52"/>
     <mergeCell ref="AE44:AE46"/>
@@ -9078,17 +9090,21 @@
     <mergeCell ref="AE32:AE34"/>
     <mergeCell ref="AE24:AE26"/>
     <mergeCell ref="P26:R26"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="I13:K13"/>
-    <mergeCell ref="L26:N26"/>
-    <mergeCell ref="P23:R23"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="C6:C8"/>
-    <mergeCell ref="F9:F11"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="O3:S4"/>
-    <mergeCell ref="F21:F23"/>
+    <mergeCell ref="C50:C52"/>
+    <mergeCell ref="C44:C46"/>
+    <mergeCell ref="C38:C40"/>
+    <mergeCell ref="C32:C34"/>
+    <mergeCell ref="C24:C26"/>
+    <mergeCell ref="AC4:AE4"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="Y41:Y43"/>
+    <mergeCell ref="Y15:Y17"/>
+    <mergeCell ref="V28:V30"/>
+    <mergeCell ref="P34:R34"/>
+    <mergeCell ref="T26:V26"/>
+    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="I41:I43"/>
+    <mergeCell ref="I15:I17"/>
   </mergeCells>
   <conditionalFormatting sqref="P26:R26">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -9216,24 +9232,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:50" s="111" customFormat="1" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="203" t="s">
+      <c r="A1" s="204" t="s">
         <v>925</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="204"/>
-      <c r="E1" s="204"/>
-      <c r="F1" s="205"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="205"/>
+      <c r="E1" s="205"/>
+      <c r="F1" s="206"/>
     </row>
     <row r="2" spans="1:50" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="213" t="s">
+      <c r="A2" s="214" t="s">
         <v>924</v>
       </c>
-      <c r="B2" s="213"/>
-      <c r="C2" s="213"/>
-      <c r="D2" s="213"/>
-      <c r="E2" s="213"/>
-      <c r="F2" s="213"/>
+      <c r="B2" s="214"/>
+      <c r="C2" s="214"/>
+      <c r="D2" s="214"/>
+      <c r="E2" s="214"/>
+      <c r="F2" s="214"/>
       <c r="K2" s="111"/>
       <c r="L2" s="111"/>
       <c r="M2" s="111"/>
@@ -9763,12 +9779,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="214" t="s">
+      <c r="A1" s="215" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="204"/>
-      <c r="C1" s="204"/>
-      <c r="D1" s="205"/>
+      <c r="B1" s="205"/>
+      <c r="C1" s="205"/>
+      <c r="D1" s="206"/>
       <c r="F1" s="34" t="s">
         <v>14</v>
       </c>
@@ -10480,17 +10496,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="215" t="s">
+      <c r="A1" s="216" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="216"/>
-      <c r="C1" s="216"/>
-      <c r="D1" s="216"/>
-      <c r="E1" s="216"/>
-      <c r="F1" s="216"/>
-      <c r="G1" s="216"/>
-      <c r="H1" s="216"/>
-      <c r="I1" s="216"/>
+      <c r="B1" s="217"/>
+      <c r="C1" s="217"/>
+      <c r="D1" s="217"/>
+      <c r="E1" s="217"/>
+      <c r="F1" s="217"/>
+      <c r="G1" s="217"/>
+      <c r="H1" s="217"/>
+      <c r="I1" s="217"/>
     </row>
     <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="55" t="s">
@@ -30181,17 +30197,17 @@
       <c r="BO1" t="s">
         <v>292</v>
       </c>
-      <c r="BT1" s="217" t="s">
+      <c r="BT1" s="218" t="s">
         <v>316</v>
       </c>
-      <c r="BU1" s="216"/>
-      <c r="BV1" s="216"/>
-      <c r="BX1" s="218" t="s">
+      <c r="BU1" s="217"/>
+      <c r="BV1" s="217"/>
+      <c r="BX1" s="219" t="s">
         <v>317</v>
       </c>
-      <c r="BY1" s="216"/>
-      <c r="BZ1" s="216"/>
-      <c r="CA1" s="216"/>
+      <c r="BY1" s="217"/>
+      <c r="BZ1" s="217"/>
+      <c r="CA1" s="217"/>
     </row>
     <row r="2" spans="1:79" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -32517,12 +32533,12 @@
       <c r="BV21" s="139" t="s">
         <v>340</v>
       </c>
-      <c r="BX21" s="217" t="s">
+      <c r="BX21" s="218" t="s">
         <v>341</v>
       </c>
-      <c r="BY21" s="216"/>
-      <c r="BZ21" s="216"/>
-      <c r="CA21" s="216"/>
+      <c r="BY21" s="217"/>
+      <c r="BZ21" s="217"/>
+      <c r="CA21" s="217"/>
     </row>
     <row r="22" spans="1:79" x14ac:dyDescent="0.25">
       <c r="A22" t="s">

</xml_diff>